<commit_message>
chore: stage remaining working-tree changes before PR merge
All modified files from the native-rewrite WIP that were not yet committed.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/stemacle-user-stories-status.xlsx
+++ b/docs/stemacle-user-stories-status.xlsx
@@ -567,7 +567,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="C3" s="3" t="str"/>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C4" s="3" t="str"/>
       <c r="D4" s="10" t="str"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>UI/UX hit-target pass: found and fixed 6 dead-tap-area bugs (Settings rows + icon buttons) and locked them plus overlap contracts behind tests/native-uiux.test.mjs. All suites green.</t>
+          <t>Bulletproofed all contracts: Cloudflare Worker API test suite, 3 separation-server shapes pinned+documented, web↔core DSP parity guards, and decommissioned the dead Electron/Capacitor/SwiftPM-macOS CI/release cluster (CI now honest+green).</t>
         </is>
       </c>
       <c r="C6" s="3" t="str"/>
@@ -642,7 +642,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="B12" s="14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O71"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -5961,6 +5961,391 @@
       <c r="O71" s="20" t="inlineStr">
         <is>
           <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-001</t>
+        </is>
+      </c>
+      <c r="B72" s="20" t="inlineStr">
+        <is>
+          <t>Cloudflare</t>
+        </is>
+      </c>
+      <c r="C72" s="20" t="inlineStr">
+        <is>
+          <t>Separation API</t>
+        </is>
+      </c>
+      <c r="D72" s="20" t="inlineStr">
+        <is>
+          <t>Edge Worker HTTP contract</t>
+        </is>
+      </c>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>As a future hosted-Demucs client, the edge Worker behaves predictably and never lies about having a GPU/Demucs backend it lacks.</t>
+        </is>
+      </c>
+      <c r="F72" s="20" t="inlineStr">
+        <is>
+          <t>GET /+/healthz healthy; /capabilities discloses demucsOnCloudflareEdge:false + currentBackend:cloudflare_queue_no_gpu_consumer; /quote bounded+clamped; /separate 503-without-bindings, 415-non-JSON, 202-with-bindings (job_id+queue.send+R2.put); /jobs/:uuid 404-unknown, malformed→not_found; OPTIONS 204 CORS.</t>
+        </is>
+      </c>
+      <c r="G72" s="20" t="inlineStr">
+        <is>
+          <t>cloudflare/stemacle-api-worker.js; tests/cloudflare-api.test.mjs</t>
+        </is>
+      </c>
+      <c r="H72" s="20" t="inlineStr">
+        <is>
+          <t>Automated behavioral tests</t>
+        </is>
+      </c>
+      <c r="I72" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass</t>
+        </is>
+      </c>
+      <c r="J72" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/cloudflare-api.test.mjs</t>
+        </is>
+      </c>
+      <c r="K72" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 14 behavioral tests (verified non-vacuous); live deployment matches.</t>
+        </is>
+      </c>
+      <c r="L72" s="20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M72" s="20" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="N72" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 14 behavioral tests against the worker handler.</t>
+        </is>
+      </c>
+      <c r="O72" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-002</t>
+        </is>
+      </c>
+      <c r="B73" s="20" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="C73" s="20" t="inlineStr">
+        <is>
+          <t>Pipelines</t>
+        </is>
+      </c>
+      <c r="D73" s="20" t="inlineStr">
+        <is>
+          <t>Honest, green CI workflows</t>
+        </is>
+      </c>
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>As a contributor, CI validates the surfaces that actually exist and does not reference deleted ones.</t>
+        </is>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
+        <is>
+          <t>pages.yml verifies real site+native files (no native/electron, native/index.html, native/ios, capacitor) and drops the broken native:prepare; release.yml runs the test gate on tags without the dead macOS-DMG build. Locked by stem-player.test.mjs honest-contract guards.</t>
+        </is>
+      </c>
+      <c r="G73" s="20" t="inlineStr">
+        <is>
+          <t>.github/workflows/pages.yml; .github/workflows/release.yml; tests/stem-player.test.mjs</t>
+        </is>
+      </c>
+      <c r="H73" s="20" t="inlineStr">
+        <is>
+          <t>Automated guard tests</t>
+        </is>
+      </c>
+      <c r="I73" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass</t>
+        </is>
+      </c>
+      <c r="J73" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/stem-player.test.mjs</t>
+        </is>
+      </c>
+      <c r="K73" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: CI no longer references deleted surfaces; npm test 142/142.</t>
+        </is>
+      </c>
+      <c r="L73" s="20" t="inlineStr">
+        <is>
+          <t>ERR-008</t>
+        </is>
+      </c>
+      <c r="M73" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="N73" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: honest-CI guards green; npm test 142/142.</t>
+        </is>
+      </c>
+      <c r="O73" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-003</t>
+        </is>
+      </c>
+      <c r="B74" s="20" t="inlineStr">
+        <is>
+          <t>Repo</t>
+        </is>
+      </c>
+      <c r="C74" s="20" t="inlineStr">
+        <is>
+          <t>Cleanup</t>
+        </is>
+      </c>
+      <c r="D74" s="20" t="inlineStr">
+        <is>
+          <t>Dead macOS/Electron/Capacitor release cluster removed</t>
+        </is>
+      </c>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>As a new agent, package.json + scripts reflect reality so I am not misled into a dead toolchain.</t>
+        </is>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
+        <is>
+          <t>Removed electron-builder build block, macos:*/native:prepare scripts, scripts/{prepare-native,package-macos}.mjs; package.json scripts carry no electron/capacitor/native-macos references; the lying green macOS-DMG release test was replaced with an honest decommission guard.</t>
+        </is>
+      </c>
+      <c r="G74" s="20" t="inlineStr">
+        <is>
+          <t>package.json; scripts/; tests/stem-player.test.mjs</t>
+        </is>
+      </c>
+      <c r="H74" s="20" t="inlineStr">
+        <is>
+          <t>Automated guard tests</t>
+        </is>
+      </c>
+      <c r="I74" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass</t>
+        </is>
+      </c>
+      <c r="J74" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/stem-player.test.mjs</t>
+        </is>
+      </c>
+      <c r="K74" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: honest release/package contract guard green.</t>
+        </is>
+      </c>
+      <c r="L74" s="20" t="inlineStr">
+        <is>
+          <t>ERR-008</t>
+        </is>
+      </c>
+      <c r="M74" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="N74" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: honest release/package contract guard green.</t>
+        </is>
+      </c>
+      <c r="O74" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-004</t>
+        </is>
+      </c>
+      <c r="B75" s="20" t="inlineStr">
+        <is>
+          <t>Cross-surface</t>
+        </is>
+      </c>
+      <c r="C75" s="20" t="inlineStr">
+        <is>
+          <t>Separation contracts</t>
+        </is>
+      </c>
+      <c r="D75" s="20" t="inlineStr">
+        <is>
+          <t>Three server shapes pinned + documented</t>
+        </is>
+      </c>
+      <c r="E75" s="20" t="inlineStr">
+        <is>
+          <t>As an integrator, the FastAPI server, Swift client, and Cloudflare worker contracts are explicit so I never confuse them.</t>
+        </is>
+      </c>
+      <c r="F75" s="20" t="inlineStr">
+        <is>
+          <t>docs/SEPARATION_CONTRACTS.md documents all three; a guard pins that the Swift client speaks the FastAPI contract (routes, fields, multipart, stems) and that the Cloudflare worker is deliberately distinct (JSON+R2, no per-stem WAV route).</t>
+        </is>
+      </c>
+      <c r="G75" s="20" t="inlineStr">
+        <is>
+          <t>docs/SEPARATION_CONTRACTS.md; tests/separation-contracts.test.mjs</t>
+        </is>
+      </c>
+      <c r="H75" s="20" t="inlineStr">
+        <is>
+          <t>Automated cross-contract tests</t>
+        </is>
+      </c>
+      <c r="I75" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass</t>
+        </is>
+      </c>
+      <c r="J75" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/separation-contracts.test.mjs</t>
+        </is>
+      </c>
+      <c r="K75" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 6 cross-contract guards green.</t>
+        </is>
+      </c>
+      <c r="L75" s="20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M75" s="20" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="N75" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 6 cross-contract guards green.</t>
+        </is>
+      </c>
+      <c r="O75" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-005</t>
+        </is>
+      </c>
+      <c r="B76" s="20" t="inlineStr">
+        <is>
+          <t>Cross-surface</t>
+        </is>
+      </c>
+      <c r="C76" s="20" t="inlineStr">
+        <is>
+          <t>DSP parity</t>
+        </is>
+      </c>
+      <c r="D76" s="20" t="inlineStr">
+        <is>
+          <t>Web↔Rust core parity for soft crossover + NaN guard</t>
+        </is>
+      </c>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>As a maintainer, the bass/melody crossover and BPM NaN guard cannot drift between the web gold master and the Rust core.</t>
+        </is>
+      </c>
+      <c r="F76" s="20" t="inlineStr">
+        <is>
+          <t>Source-parity guards assert web app/index.html and native/core share the 220/380 Hz band, the 0.5+0.5cos(PI t) crossfade, the is-finite BPM fallback to 120, and (60/bpm)*BEATS_PER_MEASURE — the two pieces not covered by golden vectors.</t>
+        </is>
+      </c>
+      <c r="G76" s="20" t="inlineStr">
+        <is>
+          <t>app/index.html; native/core/stemacle-dsp/src/{hpss,loops,tempo}.rs; tests/dsp-parity.test.mjs</t>
+        </is>
+      </c>
+      <c r="H76" s="20" t="inlineStr">
+        <is>
+          <t>Automated parity tests</t>
+        </is>
+      </c>
+      <c r="I76" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass</t>
+        </is>
+      </c>
+      <c r="J76" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/dsp-parity.test.mjs</t>
+        </is>
+      </c>
+      <c r="K76" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 5 parity guards (verified non-vacuous).</t>
+        </is>
+      </c>
+      <c r="L76" s="20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="M76" s="20" t="inlineStr">
+        <is>
+          <t>Not Applicable</t>
+        </is>
+      </c>
+      <c r="N76" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: 5 parity guards green.</t>
+        </is>
+      </c>
+      <c r="O76" s="20" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -5991,7 +6376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6463,6 +6848,63 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>ERR-008</t>
+        </is>
+      </c>
+      <c r="B9" s="20" t="inlineStr">
+        <is>
+          <t>CTRL-002; CTRL-003</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>CI</t>
+        </is>
+      </c>
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>Logistical</t>
+        </is>
+      </c>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>CI workflows + package.json referenced surfaces deleted in the native rewrite (CI was RED)</t>
+        </is>
+      </c>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>pages.yml asserted 5 deleted files exist (native/index.html, native/electron/main.cjs, native/ios/*, capacitor.config.json) and ran a broken native:prepare (copies the gone native/index.html); release.yml built a macOS DMG from the gone native/macos via electron-builder; a green test in stem-player.test.mjs locked the dead pipeline.</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>The native rewrite deleted native/electron, native/ios (Capacitor), native/macos (SwiftPM) and the native-bundle shell, but the CI/scripts/tests/package.json referencing them were never updated.</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
+        <is>
+          <t>Decommissioned the cluster: cleaned package.json (no build block/main/electron+capacitor deps/dead scripts), deleted scripts/{prepare-native,package-macos,serve-native,desktop-dispatch}.mjs, made pages.yml/release.yml honest, and replaced the lying macOS-DMG test with honest decommission guards. Removed dead test helpers that read gone files.</t>
+        </is>
+      </c>
+      <c r="K9" s="20" t="inlineStr">
+        <is>
+          <t>Retested Pass: npm test 142/142; both Apple targets BUILD SUCCEEDED.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="H2:H5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -6479,7 +6921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7014,6 +7456,80 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>RUN-015</t>
+        </is>
+      </c>
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C16" s="20" t="inlineStr">
+        <is>
+          <t>Contract hardening: Cloudflare worker + cross-contract + DSP parity</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>node --test tests/{cloudflare-api,separation-contracts,dsp-parity}.test.mjs</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>14 worker + 6 cross-contract + 5 DSP-parity guards; non-vacuous checks done. Pins the Cloudflare API, the 3 server shapes, and web↔core DSP.</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>RUN-016</t>
+        </is>
+      </c>
+      <c r="B17" s="20" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="C17" s="20" t="inlineStr">
+        <is>
+          <t>CI/release decommission + honest guards + full suite</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>npm test; cargo test core; xcodebuild macOS+iOS</t>
+        </is>
+      </c>
+      <c r="E17" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>npm test 142/142; Rust core 36 lib + 4 golden + 3 ffi; StemacleKit swift 38; both Apple targets BUILD SUCCEEDED. CI no longer references deleted surfaces.</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>